<commit_message>
new rhubarb template - kits
</commit_message>
<xml_diff>
--- a/Rhubarb_7_1_A.xlsx
+++ b/Rhubarb_7_1_A.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1436" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1460" uniqueCount="471">
   <si>
     <t>UP</t>
   </si>
@@ -1434,6 +1434,27 @@
   </si>
   <si>
     <t>7</t>
+  </si>
+  <si>
+    <t>AQ1153KIT</t>
+  </si>
+  <si>
+    <t>Cabin Air Filter - Kit (includes tool and new seals)</t>
+  </si>
+  <si>
+    <t>Filtro de aire de cabina - Kit (incluye herramienta y sellos nuevos)</t>
+  </si>
+  <si>
+    <t>AQ1053</t>
+  </si>
+  <si>
+    <t>ACME Filters</t>
+  </si>
+  <si>
+    <t>CatchAll PRO</t>
+  </si>
+  <si>
+    <t>BCDE</t>
   </si>
 </sst>
 </file>
@@ -6000,7 +6021,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:U7"/>
+  <dimension ref="A1:U8"/>
   <sheetFormatPr defaultColWidth="11.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -6304,7 +6325,7 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>186</v>
+        <v>464</v>
       </c>
       <c r="B6" s="3">
         <v>6832</v>
@@ -6313,7 +6334,7 @@
         <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>0</v>
@@ -6353,7 +6374,7 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B7" s="3">
         <v>6832</v>
@@ -6362,7 +6383,7 @@
         <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>0</v>
@@ -6377,13 +6398,13 @@
         <v>51</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="M7" s="3">
         <v>1</v>
@@ -6399,6 +6420,55 @@
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>187</v>
+      </c>
+      <c r="B8" s="3">
+        <v>6832</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
+        <v>1</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="M8" s="3">
+        <v>1</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6412,7 +6482,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.5703125" customWidth="1"/>
-    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="2" max="2" width="77.42578125" customWidth="1"/>
     <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
   </cols>
@@ -6538,10 +6608,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>185</v>
+        <v>464</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>418</v>
+        <v>465</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>53</v>
@@ -6555,10 +6625,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>185</v>
+        <v>464</v>
       </c>
       <c r="B9" s="34" t="s">
-        <v>417</v>
+        <v>466</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>53</v>
@@ -7527,24 +7597,26 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:N4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="27.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.85546875" customWidth="1"/>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="21.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
@@ -7552,82 +7624,134 @@
         <v>46</v>
       </c>
       <c r="C1" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>456</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="E1" s="7" t="s">
         <v>457</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>455</v>
       </c>
-      <c r="G1" s="8" t="s">
-        <v>459</v>
-      </c>
-      <c r="H1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>458</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>450</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="K1" s="5" t="s">
         <v>451</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="L1" s="22" t="s">
         <v>452</v>
       </c>
-      <c r="L1" s="22" t="s">
+      <c r="M1" s="22" t="s">
         <v>453</v>
       </c>
-      <c r="M1" s="22" t="s">
+      <c r="N1" s="22" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>185</v>
+        <v>464</v>
       </c>
       <c r="B2" t="s">
         <v>460</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G2" t="s">
+        <v>52</v>
+      </c>
+      <c r="H2">
+        <v>6832</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2" t="s">
+        <v>467</v>
+      </c>
+      <c r="K2" t="s">
+        <v>78</v>
+      </c>
+      <c r="L2" t="s">
+        <v>468</v>
+      </c>
+      <c r="M2" t="s">
+        <v>470</v>
+      </c>
+      <c r="N2" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>185</v>
+        <v>464</v>
       </c>
       <c r="B3" t="s">
         <v>461</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>185</v>
+        <v>464</v>
       </c>
       <c r="B4" t="s">
         <v>462</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4">
         <v>2</v>
       </c>
-      <c r="D4" t="s">
-        <v>1</v>
+      <c r="E4" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="I4">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>